<commit_message>
Deliverable picker: source the model, add four formats; rename Plot Thickens
Footer reworked from a figure-only credit into a knowledge-translation
framing that names the scholarship the picker's three axes actually rest
on: Tabak et al. (2013) for the audience subgroups, COSCA (2024) for the
objectives, and Duarte / Nussbaumer Knaflic / Segel and Heer for the
method, framed by Lavis et al. (2003). All were already footnoted in the
maintainer's own Trends chapter; the page just credited the figures, not
the scholarship under them.

Adds four deliverables from practice (Workshop and Webinar kept separate,
Research Poster, Op-ed or Commentary), taking the workbook to 21 formats;
all use existing families so GROUP_COLORS is unchanged. Validated by
build_format.R (9/9 checks) and the page's own evaluate() across fits /
adapt-for-reach / ruled-out scenarios.

Publications section "The Four Threads" renamed to "The Plot Thickens".

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/formatpicker/data/delivery_formats.xlsx
+++ b/formatpicker/data/delivery_formats.xlsx
@@ -799,7 +799,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2003,6 +2003,274 @@
         </is>
       </c>
       <c r="M18" t="inlineStr">
+        <is>
+          <t>Added from practice (2026); not in the Trends Fig. 2 tree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WORKSHOP</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>A hands-on working session where the group learns or decides by doing, with you facilitating.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Internal;Both</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Generalist;Colleague;Expert</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Inform/Explain;Support a Decision</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Building data literacy, walking a team through a method, or facilitating a session where the group works through the data with you.</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>A one-way announcement, or anything that must travel afterward without a facilitator.</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Half a day to a full day, in person or small-group virtual.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Added from practice (2026); not in the Trends Fig. 2 tree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WEBINAR</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Webinar</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>A live online session that carries a talk to a broad, registered audience.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Both;External</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Novice;Generalist;Colleague;Expert</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Inform/Explain;Raise Awareness</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Reaching people across locations at once, introducing a topic, or presenting to partners and the public without travel.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Deep hands-on work, or a small internal group a meeting would serve better.</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>45 to 60 minutes, live, often recorded.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Added from practice (2026); not in the Trends Fig. 2 tree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>POSTER</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Research Poster</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>A single visual board that carries one finding at a conference or event.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Both;External</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Generalist;Colleague;Expert</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Inform/Explain;Raise Awareness</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Summarizing a study for a professional audience, or presenting where a full talk is not on offer.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Detail-heavy reporting, or any audience that will not stand and read.</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>One board, roughly 36 by 48 inches.</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Added from practice (2026); not in the Trends Fig. 2 tree.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>OPED</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Op-ed or Commentary</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Outreach &amp; media</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>A short authored argument placed in an outlet your audience already reads.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Novice;Generalist</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Persuade/Advocate;Raise Awareness;Inform/Explain</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Short</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Making a case in your own voice, or putting a finding in front of readers who will not seek out a report.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Neutral documentation, or a full account of methods and caveats.</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>600 to 800 words.</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
         <is>
           <t>Added from practice (2026); not in the Trends Fig. 2 tree.</t>
         </is>

</xml_diff>